<commit_message>
Pre Market Tue 2026-06-16
</commit_message>
<xml_diff>
--- a/pre-market/Pre Market 2026-06-16.xlsx
+++ b/pre-market/Pre Market 2026-06-16.xlsx
@@ -459,7 +459,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7554,55</t>
+          <t>7554,28</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -476,7 +476,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30524,05</t>
+          <t>30543,92</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2965,12</t>
+          <t>2965,09</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>51671,84</t>
+          <t>51671,04</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4321,08</t>
+          <t>4309,68</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>70,21</t>
+          <t>69,98</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1775,60</t>
+          <t>1772,10</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>83,77</t>
+          <t>83,17</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>66513,42</t>
+          <t>66442,91</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1817,93</t>
+          <t>1815,98</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-9,05%</t>
+          <t>-8,37%</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>7555,17</t>
+          <t>7554,29</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>

</xml_diff>